<commit_message>
docs: add sliding caliper reading animation and update update date in index.html
</commit_message>
<xml_diff>
--- a/OI/TQ_2026 CQPM Technicien qualité - Bourges 5-6 Novembre  2026/V3_Formation_Salaries/Flash_mesure_TQ6.xlsx
+++ b/OI/TQ_2026 CQPM Technicien qualité - Bourges 5-6 Novembre  2026/V3_Formation_Salaries/Flash_mesure_TQ6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/TQ_2026 CQPM Technicien qualité - Bourges 5-6 Novembre  2026/V3_Formation_Salaries/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="11_F9490EB66F15501B7E4EA62C01BC0C8D3914521F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36243C6B-D283-47D2-AA5F-09F2A7B5626A}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_F9490EB66F15501B7E4EA62C01BC0C8D3914521F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E23168E-DAA3-46DF-9DFE-4F96DAB1CF19}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,22 +427,9 @@
   </cellStyleXfs>
   <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -470,7 +457,6 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -509,6 +495,20 @@
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,255 +794,255 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="1:10" ht="26.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
     </row>
     <row r="9" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+      <c r="A10" s="5">
         <v>1</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="16">
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="9">
         <f t="shared" ref="J10:J15" si="0">COUNT(D10,E10,F10,G10,H10,I10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12">
+      <c r="A11" s="5">
         <v>2</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="16">
+      <c r="B11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12">
+      <c r="A12" s="5">
         <v>3</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="16">
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12">
+      <c r="A13" s="5">
         <v>4</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="16">
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12">
+      <c r="A14" s="5">
         <v>5</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="16">
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12">
+      <c r="A15" s="5">
         <v>6</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="16">
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="18" t="str">
+      <c r="J16" s="11" t="str">
         <f>SUM(J10:J15)&amp;" / 36"</f>
         <v>0 / 36</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="29"/>
+      <c r="J18" s="29"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1081,426 +1081,426 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="12" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="13" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="21" t="s">
+      <c r="B3" s="35"/>
+      <c r="C3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="3" t="str">
+      <c r="E3" s="36" t="str">
         <f>Saisie!J16&amp;" mesures saisies"</f>
         <v>0 / 36 mesures saisies</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
     </row>
     <row r="5" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25">
+      <c r="A6" s="17">
         <f>IF(Saisie!B10="",1,1&amp;" · "&amp;Saisie!B10)</f>
         <v>1</v>
       </c>
-      <c r="B6" s="26" t="str">
+      <c r="B6" s="18" t="str">
         <f>IF(Saisie!D10="","",IF($C$3="OUI",Saisie!D10,"✓"))</f>
         <v/>
       </c>
-      <c r="C6" s="26" t="str">
+      <c r="C6" s="18" t="str">
         <f>IF(Saisie!E10="","",IF($C$3="OUI",Saisie!E10,"✓"))</f>
         <v/>
       </c>
-      <c r="D6" s="26" t="str">
+      <c r="D6" s="18" t="str">
         <f>IF(Saisie!F10="","",IF($C$3="OUI",Saisie!F10,"✓"))</f>
         <v/>
       </c>
-      <c r="E6" s="26" t="str">
+      <c r="E6" s="18" t="str">
         <f>IF(Saisie!G10="","",IF($C$3="OUI",Saisie!G10,"✓"))</f>
         <v/>
       </c>
-      <c r="F6" s="26" t="str">
+      <c r="F6" s="18" t="str">
         <f>IF(Saisie!H10="","",IF($C$3="OUI",Saisie!H10,"✓"))</f>
         <v/>
       </c>
-      <c r="G6" s="27" t="str">
+      <c r="G6" s="19" t="str">
         <f>IF(Saisie!I10="","",IF($C$3="OUI",Saisie!I10,"✓"))</f>
         <v/>
       </c>
-      <c r="H6" s="28" t="str">
+      <c r="H6" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D10:H10)=5),ROUND(MAX(Saisie!D10:H10)-MIN(Saisie!D10:H10),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25">
+      <c r="A7" s="17">
         <f>IF(Saisie!B11="",2,2&amp;" · "&amp;Saisie!B11)</f>
         <v>2</v>
       </c>
-      <c r="B7" s="26" t="str">
+      <c r="B7" s="18" t="str">
         <f>IF(Saisie!D11="","",IF($C$3="OUI",Saisie!D11,"✓"))</f>
         <v/>
       </c>
-      <c r="C7" s="26" t="str">
+      <c r="C7" s="18" t="str">
         <f>IF(Saisie!E11="","",IF($C$3="OUI",Saisie!E11,"✓"))</f>
         <v/>
       </c>
-      <c r="D7" s="26" t="str">
+      <c r="D7" s="18" t="str">
         <f>IF(Saisie!F11="","",IF($C$3="OUI",Saisie!F11,"✓"))</f>
         <v/>
       </c>
-      <c r="E7" s="26" t="str">
+      <c r="E7" s="18" t="str">
         <f>IF(Saisie!G11="","",IF($C$3="OUI",Saisie!G11,"✓"))</f>
         <v/>
       </c>
-      <c r="F7" s="26" t="str">
+      <c r="F7" s="18" t="str">
         <f>IF(Saisie!H11="","",IF($C$3="OUI",Saisie!H11,"✓"))</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="str">
+      <c r="G7" s="19" t="str">
         <f>IF(Saisie!I11="","",IF($C$3="OUI",Saisie!I11,"✓"))</f>
         <v/>
       </c>
-      <c r="H7" s="28" t="str">
+      <c r="H7" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D11:H11)=5),ROUND(MAX(Saisie!D11:H11)-MIN(Saisie!D11:H11),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25">
+      <c r="A8" s="17">
         <f>IF(Saisie!B12="",3,3&amp;" · "&amp;Saisie!B12)</f>
         <v>3</v>
       </c>
-      <c r="B8" s="26" t="str">
+      <c r="B8" s="18" t="str">
         <f>IF(Saisie!D12="","",IF($C$3="OUI",Saisie!D12,"✓"))</f>
         <v/>
       </c>
-      <c r="C8" s="26" t="str">
+      <c r="C8" s="18" t="str">
         <f>IF(Saisie!E12="","",IF($C$3="OUI",Saisie!E12,"✓"))</f>
         <v/>
       </c>
-      <c r="D8" s="26" t="str">
+      <c r="D8" s="18" t="str">
         <f>IF(Saisie!F12="","",IF($C$3="OUI",Saisie!F12,"✓"))</f>
         <v/>
       </c>
-      <c r="E8" s="26" t="str">
+      <c r="E8" s="18" t="str">
         <f>IF(Saisie!G12="","",IF($C$3="OUI",Saisie!G12,"✓"))</f>
         <v/>
       </c>
-      <c r="F8" s="26" t="str">
+      <c r="F8" s="18" t="str">
         <f>IF(Saisie!H12="","",IF($C$3="OUI",Saisie!H12,"✓"))</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="str">
+      <c r="G8" s="19" t="str">
         <f>IF(Saisie!I12="","",IF($C$3="OUI",Saisie!I12,"✓"))</f>
         <v/>
       </c>
-      <c r="H8" s="28" t="str">
+      <c r="H8" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D12:H12)=5),ROUND(MAX(Saisie!D12:H12)-MIN(Saisie!D12:H12),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25">
+      <c r="A9" s="17">
         <f>IF(Saisie!B13="",4,4&amp;" · "&amp;Saisie!B13)</f>
         <v>4</v>
       </c>
-      <c r="B9" s="26" t="str">
+      <c r="B9" s="18" t="str">
         <f>IF(Saisie!D13="","",IF($C$3="OUI",Saisie!D13,"✓"))</f>
         <v/>
       </c>
-      <c r="C9" s="26" t="str">
+      <c r="C9" s="18" t="str">
         <f>IF(Saisie!E13="","",IF($C$3="OUI",Saisie!E13,"✓"))</f>
         <v/>
       </c>
-      <c r="D9" s="26" t="str">
+      <c r="D9" s="18" t="str">
         <f>IF(Saisie!F13="","",IF($C$3="OUI",Saisie!F13,"✓"))</f>
         <v/>
       </c>
-      <c r="E9" s="26" t="str">
+      <c r="E9" s="18" t="str">
         <f>IF(Saisie!G13="","",IF($C$3="OUI",Saisie!G13,"✓"))</f>
         <v/>
       </c>
-      <c r="F9" s="26" t="str">
+      <c r="F9" s="18" t="str">
         <f>IF(Saisie!H13="","",IF($C$3="OUI",Saisie!H13,"✓"))</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="str">
+      <c r="G9" s="19" t="str">
         <f>IF(Saisie!I13="","",IF($C$3="OUI",Saisie!I13,"✓"))</f>
         <v/>
       </c>
-      <c r="H9" s="28" t="str">
+      <c r="H9" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D13:H13)=5),ROUND(MAX(Saisie!D13:H13)-MIN(Saisie!D13:H13),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25">
+      <c r="A10" s="17">
         <f>IF(Saisie!B14="",5,5&amp;" · "&amp;Saisie!B14)</f>
         <v>5</v>
       </c>
-      <c r="B10" s="26" t="str">
+      <c r="B10" s="18" t="str">
         <f>IF(Saisie!D14="","",IF($C$3="OUI",Saisie!D14,"✓"))</f>
         <v/>
       </c>
-      <c r="C10" s="26" t="str">
+      <c r="C10" s="18" t="str">
         <f>IF(Saisie!E14="","",IF($C$3="OUI",Saisie!E14,"✓"))</f>
         <v/>
       </c>
-      <c r="D10" s="26" t="str">
+      <c r="D10" s="18" t="str">
         <f>IF(Saisie!F14="","",IF($C$3="OUI",Saisie!F14,"✓"))</f>
         <v/>
       </c>
-      <c r="E10" s="26" t="str">
+      <c r="E10" s="18" t="str">
         <f>IF(Saisie!G14="","",IF($C$3="OUI",Saisie!G14,"✓"))</f>
         <v/>
       </c>
-      <c r="F10" s="26" t="str">
+      <c r="F10" s="18" t="str">
         <f>IF(Saisie!H14="","",IF($C$3="OUI",Saisie!H14,"✓"))</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="str">
+      <c r="G10" s="19" t="str">
         <f>IF(Saisie!I14="","",IF($C$3="OUI",Saisie!I14,"✓"))</f>
         <v/>
       </c>
-      <c r="H10" s="28" t="str">
+      <c r="H10" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D14:H14)=5),ROUND(MAX(Saisie!D14:H14)-MIN(Saisie!D14:H14),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25">
+      <c r="A11" s="17">
         <f>IF(Saisie!B15="",6,6&amp;" · "&amp;Saisie!B15)</f>
         <v>6</v>
       </c>
-      <c r="B11" s="26" t="str">
+      <c r="B11" s="18" t="str">
         <f>IF(Saisie!D15="","",IF($C$3="OUI",Saisie!D15,"✓"))</f>
         <v/>
       </c>
-      <c r="C11" s="26" t="str">
+      <c r="C11" s="18" t="str">
         <f>IF(Saisie!E15="","",IF($C$3="OUI",Saisie!E15,"✓"))</f>
         <v/>
       </c>
-      <c r="D11" s="26" t="str">
+      <c r="D11" s="18" t="str">
         <f>IF(Saisie!F15="","",IF($C$3="OUI",Saisie!F15,"✓"))</f>
         <v/>
       </c>
-      <c r="E11" s="26" t="str">
+      <c r="E11" s="18" t="str">
         <f>IF(Saisie!G15="","",IF($C$3="OUI",Saisie!G15,"✓"))</f>
         <v/>
       </c>
-      <c r="F11" s="26" t="str">
+      <c r="F11" s="18" t="str">
         <f>IF(Saisie!H15="","",IF($C$3="OUI",Saisie!H15,"✓"))</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="str">
+      <c r="G11" s="19" t="str">
         <f>IF(Saisie!I15="","",IF($C$3="OUI",Saisie!I15,"✓"))</f>
         <v/>
       </c>
-      <c r="H11" s="28" t="str">
+      <c r="H11" s="20" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D15:H15)=5),ROUND(MAX(Saisie!D15:H15)-MIN(Saisie!D15:H15),3),"")</f>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="30" t="str">
+      <c r="B12" s="22" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D10:D15)&gt;=2),ROUND(MAX(Saisie!D10:D15)-MIN(Saisie!D10:D15),3),"")</f>
         <v/>
       </c>
-      <c r="C12" s="30" t="str">
+      <c r="C12" s="22" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!E10:E15)&gt;=2),ROUND(MAX(Saisie!E10:E15)-MIN(Saisie!E10:E15),3),"")</f>
         <v/>
       </c>
-      <c r="D12" s="30" t="str">
+      <c r="D12" s="22" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!F10:F15)&gt;=2),ROUND(MAX(Saisie!F10:F15)-MIN(Saisie!F10:F15),3),"")</f>
         <v/>
       </c>
-      <c r="E12" s="30" t="str">
+      <c r="E12" s="22" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!G10:G15)&gt;=2),ROUND(MAX(Saisie!G10:G15)-MIN(Saisie!G10:G15),3),"")</f>
         <v/>
       </c>
-      <c r="F12" s="30" t="str">
+      <c r="F12" s="22" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!H10:H15)&gt;=2),ROUND(MAX(Saisie!H10:H15)-MIN(Saisie!H10:H15),3),"")</f>
         <v/>
       </c>
-      <c r="G12" s="31" t="str">
+      <c r="G12" s="23" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!I10:I15)&gt;=2),ROUND(MAX(Saisie!I10:I15)-MIN(Saisie!I10:I15),3),"")</f>
         <v/>
       </c>
-      <c r="H12" s="32"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="25">
         <f>COUNT(Saisie!D10:D15)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="25">
         <f>COUNT(Saisie!E10:E15)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="25">
         <f>COUNT(Saisie!F10:F15)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="25">
         <f>COUNT(Saisie!G10:G15)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="25">
         <f>COUNT(Saisie!H10:H15)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="33">
+      <c r="G13" s="25">
         <f>COUNT(Saisie!I10:I15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="34" t="str">
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="26" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!D10:D15)&gt;=2),ROUND(MAX(Saisie!D10:D15)-MIN(Saisie!D10:D15),3),"")</f>
         <v/>
       </c>
-      <c r="H16" s="35" t="s">
+      <c r="H16" s="27" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="36" t="str">
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="28" t="str">
         <f>IF(AND($C$3="OUI",COUNT(Saisie!I10:I15)&gt;=2),ROUND(MAX(Saisie!I10:I15)-MIN(Saisie!I10:I15),3),"")</f>
         <v/>
       </c>
-      <c r="H17" s="35" t="s">
+      <c r="H17" s="27" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="36" t="str">
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="28" t="str">
         <f>IF(AND($C$3="OUI",COUNT(B12:F12)&gt;=1),AVERAGE(B12:F12),"")</f>
         <v/>
       </c>
-      <c r="H18" s="35" t="s">
+      <c r="H18" s="27" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="36" t="str">
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="28" t="str">
         <f>IF(AND($C$3="OUI",COUNT(H6:H11)&gt;=1),AVERAGE(H6:H11),"")</f>
         <v/>
       </c>
-      <c r="H19" s="35" t="s">
+      <c r="H19" s="27" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="B21" s="34"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>